<commit_message>
working on 2.0.0 doc
</commit_message>
<xml_diff>
--- a/dialbb/no_code/templates/en/dst-knowledge.xlsx
+++ b/dialbb/no_code/templates/en/dst-knowledge.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nakano\system\dialbb\dialbb-next\sample_apps\dst_stn_en\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nakano\system\dialbb\dialbb-next\dialbb\no_code\templates\en\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16B7C91F-A738-4EB9-A788-43C36527A310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{695B8ECE-BD37-43E6-B383-190AE1800881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C3566FB2-A815-41D8-9347-99D11DD601B4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C3566FB2-A815-41D8-9347-99D11DD601B4}"/>
   </bookViews>
   <sheets>
     <sheet name="dialogues" sheetId="2" r:id="rId1"/>
@@ -94,10 +94,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>favorite-sandwich</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>slot name</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -144,15 +140,6 @@
   <si>
     <t>Vegetable Sandwiches, vegetable</t>
     <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>favorite-sandwich=roast beef sandwiches</t>
-  </si>
-  <si>
-    <t>favorite-sandwich=chicken salad sandwiches</t>
-  </si>
-  <si>
-    <t>user-name</t>
   </si>
   <si>
     <t>John</t>
@@ -179,14 +166,8 @@
 User: chiken salad sandwich</t>
   </si>
   <si>
-    <t>user-name=Bob</t>
-  </si>
-  <si>
     <t>System: Hi, I'm john.
 User: Hi I'm Bob.</t>
-  </si>
-  <si>
-    <t>user-name=Linda</t>
   </si>
   <si>
     <t>System: Can I have your name?
@@ -199,7 +180,25 @@
 User: Yes, I like roast beef sandwiches</t>
   </si>
   <si>
-    <t>user-name=Linda, favorite-sandwich=roast beef sandwiches</t>
+    <t>user_name=Bob</t>
+  </si>
+  <si>
+    <t>user_name=Linda</t>
+  </si>
+  <si>
+    <t>user_name</t>
+  </si>
+  <si>
+    <t>favorite_sandwich=roast beef sandwiches</t>
+  </si>
+  <si>
+    <t>favorite_sandwich=chicken salad sandwiches</t>
+  </si>
+  <si>
+    <t>user_name=Linda, favorite_sandwich=roast beef sandwiches</t>
+  </si>
+  <si>
+    <t>favorite_sandwich</t>
   </si>
 </sst>
 </file>
@@ -614,10 +613,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="30">
@@ -625,10 +624,10 @@
         <v>2</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="30">
@@ -636,10 +635,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="30">
@@ -647,43 +646,43 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="30">
       <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>39</v>
-      </c>
       <c r="C5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="30">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="60">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
         <v>42</v>
-      </c>
-      <c r="C7" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -708,7 +707,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -719,10 +718,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>4</v>
@@ -733,128 +732,128 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -862,10 +861,10 @@
         <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -873,10 +872,10 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>